<commit_message>
feat: enhance login page tests to verify visual elements and remove duplicate title
</commit_message>
<xml_diff>
--- a/base/Programação serviço de campo - Bancários.xlsx
+++ b/base/Programação serviço de campo - Bancários.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\carlo\OneDrive\Documentos\PROJETOS\Dirigentes\base\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{820B3504-8787-4F90-BF9B-60A352BE5F2E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3EF5701F-E83E-4998-9D5D-53DE9C4C4160}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Programação" sheetId="3" r:id="rId1"/>
@@ -870,15 +870,33 @@
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -895,74 +913,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="6" fillId="0" borderId="7" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="24" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="29" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="27" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="26" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="28" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -974,9 +930,53 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="25" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="27" fillId="12" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="12" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="10" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1657,42 +1657,42 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="45" customHeight="1">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="36" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="31"/>
-      <c r="C1" s="31"/>
-      <c r="D1" s="31"/>
+      <c r="B1" s="37"/>
+      <c r="C1" s="37"/>
+      <c r="D1" s="37"/>
       <c r="E1" s="18" t="s">
         <v>32</v>
       </c>
       <c r="F1" s="5"/>
     </row>
     <row r="2" spans="1:6" ht="28.5" customHeight="1">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="27"/>
-      <c r="C2" s="27"/>
-      <c r="D2" s="27"/>
-      <c r="E2" s="27"/>
+      <c r="B2" s="33"/>
+      <c r="C2" s="33"/>
+      <c r="D2" s="33"/>
+      <c r="E2" s="33"/>
       <c r="F2" s="5"/>
     </row>
     <row r="3" spans="1:6" ht="4.5" customHeight="1">
-      <c r="A3" s="28"/>
-      <c r="B3" s="29"/>
-      <c r="C3" s="29"/>
-      <c r="D3" s="29"/>
-      <c r="E3" s="29"/>
+      <c r="A3" s="34"/>
+      <c r="B3" s="35"/>
+      <c r="C3" s="35"/>
+      <c r="D3" s="35"/>
+      <c r="E3" s="35"/>
     </row>
     <row r="4" spans="1:6" ht="35.25" customHeight="1">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="24"/>
-      <c r="C4" s="24"/>
-      <c r="D4" s="24"/>
-      <c r="E4" s="24"/>
+      <c r="B4" s="31"/>
+      <c r="C4" s="31"/>
+      <c r="D4" s="31"/>
+      <c r="E4" s="31"/>
     </row>
     <row r="5" spans="1:6" ht="43.5" customHeight="1">
       <c r="A5" s="4" t="s">
@@ -1792,20 +1792,20 @@
       <c r="E10" s="3"/>
     </row>
     <row r="11" spans="1:6" ht="15" customHeight="1">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="25"/>
+      <c r="A11" s="27"/>
+      <c r="B11" s="27"/>
+      <c r="C11" s="27"/>
+      <c r="D11" s="27"/>
+      <c r="E11" s="27"/>
     </row>
     <row r="12" spans="1:6" ht="35.25" customHeight="1">
-      <c r="A12" s="33" t="s">
+      <c r="A12" s="24" t="s">
         <v>28</v>
       </c>
-      <c r="B12" s="33"/>
-      <c r="C12" s="33"/>
-      <c r="D12" s="33"/>
-      <c r="E12" s="33"/>
+      <c r="B12" s="24"/>
+      <c r="C12" s="24"/>
+      <c r="D12" s="24"/>
+      <c r="E12" s="24"/>
       <c r="F12" s="6"/>
     </row>
     <row r="13" spans="1:6" ht="39" customHeight="1">
@@ -1858,20 +1858,20 @@
       </c>
     </row>
     <row r="16" spans="1:6" ht="15" customHeight="1">
-      <c r="A16" s="25"/>
-      <c r="B16" s="25"/>
-      <c r="C16" s="25"/>
-      <c r="D16" s="25"/>
-      <c r="E16" s="25"/>
+      <c r="A16" s="27"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
     </row>
     <row r="17" spans="1:6" ht="35.25" customHeight="1">
-      <c r="A17" s="35" t="s">
+      <c r="A17" s="26" t="s">
         <v>29</v>
       </c>
-      <c r="B17" s="35"/>
-      <c r="C17" s="35"/>
-      <c r="D17" s="35"/>
-      <c r="E17" s="35"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
       <c r="F17" s="6"/>
     </row>
     <row r="18" spans="1:6" ht="39" customHeight="1">
@@ -1948,20 +1948,20 @@
       </c>
     </row>
     <row r="23" spans="1:6" ht="15" customHeight="1">
-      <c r="A23" s="25"/>
-      <c r="B23" s="25"/>
-      <c r="C23" s="25"/>
-      <c r="D23" s="25"/>
-      <c r="E23" s="25"/>
+      <c r="A23" s="27"/>
+      <c r="B23" s="27"/>
+      <c r="C23" s="27"/>
+      <c r="D23" s="27"/>
+      <c r="E23" s="27"/>
     </row>
     <row r="24" spans="1:6" ht="35.25" customHeight="1">
-      <c r="A24" s="34" t="s">
+      <c r="A24" s="25" t="s">
         <v>30</v>
       </c>
-      <c r="B24" s="34"/>
-      <c r="C24" s="34"/>
-      <c r="D24" s="34"/>
-      <c r="E24" s="34"/>
+      <c r="B24" s="25"/>
+      <c r="C24" s="25"/>
+      <c r="D24" s="25"/>
+      <c r="E24" s="25"/>
       <c r="F24" s="6"/>
     </row>
     <row r="25" spans="1:6" ht="39" customHeight="1">
@@ -2050,20 +2050,20 @@
       </c>
     </row>
     <row r="30" spans="1:6" ht="15" customHeight="1">
-      <c r="A30" s="25"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
+      <c r="A30" s="27"/>
+      <c r="B30" s="27"/>
+      <c r="C30" s="27"/>
+      <c r="D30" s="27"/>
+      <c r="E30" s="27"/>
     </row>
     <row r="31" spans="1:6" ht="35.25" customHeight="1">
-      <c r="A31" s="36" t="s">
+      <c r="A31" s="28" t="s">
         <v>44</v>
       </c>
-      <c r="B31" s="36"/>
-      <c r="C31" s="36"/>
-      <c r="D31" s="36"/>
-      <c r="E31" s="36"/>
+      <c r="B31" s="28"/>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
       <c r="F31" s="6"/>
     </row>
     <row r="32" spans="1:6" ht="39" customHeight="1">
@@ -2135,23 +2135,28 @@
       </c>
     </row>
     <row r="36" spans="1:5" ht="19.5" customHeight="1">
-      <c r="A36" s="37"/>
-      <c r="B36" s="37"/>
-      <c r="C36" s="37"/>
-      <c r="D36" s="37"/>
-      <c r="E36" s="37"/>
+      <c r="A36" s="29"/>
+      <c r="B36" s="29"/>
+      <c r="C36" s="29"/>
+      <c r="D36" s="29"/>
+      <c r="E36" s="29"/>
     </row>
     <row r="37" spans="1:5" ht="36.75" customHeight="1">
-      <c r="A37" s="32" t="s">
+      <c r="A37" s="23" t="s">
         <v>4</v>
       </c>
-      <c r="B37" s="32"/>
-      <c r="C37" s="32"/>
-      <c r="D37" s="32"/>
-      <c r="E37" s="32"/>
+      <c r="B37" s="23"/>
+      <c r="C37" s="23"/>
+      <c r="D37" s="23"/>
+      <c r="E37" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="14">
+    <mergeCell ref="A4:E4"/>
+    <mergeCell ref="A11:E11"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A3:E3"/>
+    <mergeCell ref="A1:D1"/>
     <mergeCell ref="A37:E37"/>
     <mergeCell ref="A12:E12"/>
     <mergeCell ref="A24:E24"/>
@@ -2161,11 +2166,6 @@
     <mergeCell ref="A16:E16"/>
     <mergeCell ref="A30:E30"/>
     <mergeCell ref="A36:E36"/>
-    <mergeCell ref="A4:E4"/>
-    <mergeCell ref="A11:E11"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A3:E3"/>
-    <mergeCell ref="A1:D1"/>
   </mergeCells>
   <pageMargins left="0.23622047244094491" right="0.23622047244094491" top="0.19685039370078741" bottom="0.19685039370078741" header="0.31496062992125984" footer="0.31496062992125984"/>
   <pageSetup paperSize="9" scale="65" orientation="portrait" horizontalDpi="4294967293" r:id="rId1"/>
@@ -2201,34 +2201,34 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:26" ht="40.5" customHeight="1">
-      <c r="A1" s="57" t="s">
+      <c r="A1" s="38" t="s">
         <v>52</v>
       </c>
       <c r="B1" s="39"/>
       <c r="C1" s="39"/>
       <c r="D1" s="39"/>
       <c r="E1" s="39"/>
-      <c r="F1" s="58" t="s">
+      <c r="F1" s="40" t="s">
         <v>37</v>
       </c>
       <c r="G1" s="39"/>
     </row>
     <row r="2" spans="1:26" ht="36" customHeight="1" thickBot="1">
-      <c r="A2" s="59" t="s">
+      <c r="A2" s="41" t="s">
         <v>53</v>
       </c>
-      <c r="B2" s="60"/>
-      <c r="C2" s="60"/>
-      <c r="D2" s="60"/>
-      <c r="E2" s="60"/>
-      <c r="F2" s="60"/>
-      <c r="G2" s="60"/>
+      <c r="B2" s="42"/>
+      <c r="C2" s="42"/>
+      <c r="D2" s="42"/>
+      <c r="E2" s="42"/>
+      <c r="F2" s="42"/>
+      <c r="G2" s="42"/>
     </row>
     <row r="3" spans="1:26" ht="57.75" customHeight="1">
-      <c r="A3" s="61" t="s">
+      <c r="A3" s="43" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="62"/>
+      <c r="B3" s="44"/>
       <c r="C3" s="19" t="s">
         <v>54</v>
       </c>
@@ -2265,7 +2265,7 @@
       <c r="Z3" s="22"/>
     </row>
     <row r="4" spans="1:26" ht="50.25" customHeight="1">
-      <c r="A4" s="53"/>
+      <c r="A4" s="45"/>
       <c r="B4" s="39"/>
       <c r="C4" s="39"/>
       <c r="D4" s="39"/>
@@ -2274,39 +2274,39 @@
       <c r="G4" s="39"/>
     </row>
     <row r="5" spans="1:26" ht="37.5" customHeight="1">
-      <c r="A5" s="42" t="s">
+      <c r="A5" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="63" t="s">
+      <c r="B5" s="52"/>
+      <c r="C5" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="D5" s="44" t="s">
+      <c r="D5" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="44" t="s">
+      <c r="E5" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="F5" s="44" t="s">
+      <c r="F5" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="G5" s="44" t="s">
+      <c r="G5" s="46" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="6" spans="1:26" ht="85.5" customHeight="1" thickBot="1">
-      <c r="A6" s="54">
+      <c r="A6" s="48">
         <v>1</v>
       </c>
-      <c r="B6" s="47"/>
-      <c r="C6" s="45"/>
-      <c r="D6" s="45"/>
-      <c r="E6" s="45"/>
-      <c r="F6" s="45"/>
-      <c r="G6" s="45"/>
+      <c r="B6" s="49"/>
+      <c r="C6" s="47"/>
+      <c r="D6" s="47"/>
+      <c r="E6" s="47"/>
+      <c r="F6" s="47"/>
+      <c r="G6" s="47"/>
     </row>
     <row r="7" spans="1:26" ht="36" customHeight="1">
-      <c r="A7" s="55"/>
+      <c r="A7" s="50"/>
       <c r="B7" s="39"/>
       <c r="C7" s="39"/>
       <c r="D7" s="39"/>
@@ -2315,39 +2315,39 @@
       <c r="G7" s="39"/>
     </row>
     <row r="8" spans="1:26" ht="37.5" customHeight="1">
-      <c r="A8" s="48" t="s">
+      <c r="A8" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="B8" s="43"/>
-      <c r="C8" s="49" t="s">
+      <c r="B8" s="52"/>
+      <c r="C8" s="53" t="s">
         <v>62</v>
       </c>
-      <c r="D8" s="56" t="s">
+      <c r="D8" s="54" t="s">
         <v>60</v>
       </c>
-      <c r="E8" s="50" t="s">
+      <c r="E8" s="56" t="s">
         <v>63</v>
       </c>
-      <c r="F8" s="50" t="s">
+      <c r="F8" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="G8" s="50" t="s">
+      <c r="G8" s="56" t="s">
         <v>61</v>
       </c>
     </row>
     <row r="9" spans="1:26" ht="85.5" customHeight="1" thickBot="1">
-      <c r="A9" s="52">
+      <c r="A9" s="57">
         <v>4</v>
       </c>
-      <c r="B9" s="47"/>
-      <c r="C9" s="45"/>
-      <c r="D9" s="51"/>
-      <c r="E9" s="51"/>
-      <c r="F9" s="51"/>
-      <c r="G9" s="51"/>
+      <c r="B9" s="49"/>
+      <c r="C9" s="47"/>
+      <c r="D9" s="55"/>
+      <c r="E9" s="55"/>
+      <c r="F9" s="55"/>
+      <c r="G9" s="55"/>
     </row>
     <row r="10" spans="1:26" ht="36" customHeight="1">
-      <c r="A10" s="55"/>
+      <c r="A10" s="50"/>
       <c r="B10" s="39"/>
       <c r="C10" s="39"/>
       <c r="D10" s="39"/>
@@ -2356,39 +2356,39 @@
       <c r="G10" s="39"/>
     </row>
     <row r="11" spans="1:26" ht="37.5" customHeight="1">
-      <c r="A11" s="42" t="s">
+      <c r="A11" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="B11" s="43"/>
-      <c r="C11" s="44" t="s">
+      <c r="B11" s="52"/>
+      <c r="C11" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="D11" s="44" t="s">
+      <c r="D11" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="E11" s="44" t="s">
+      <c r="E11" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="F11" s="44" t="s">
+      <c r="F11" s="46" t="s">
         <v>63</v>
       </c>
-      <c r="G11" s="44" t="s">
+      <c r="G11" s="46" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="12" spans="1:26" ht="85.5" customHeight="1" thickBot="1">
-      <c r="A12" s="54">
+      <c r="A12" s="48">
         <v>8</v>
       </c>
-      <c r="B12" s="47"/>
-      <c r="C12" s="45"/>
-      <c r="D12" s="45"/>
-      <c r="E12" s="45"/>
-      <c r="F12" s="45"/>
-      <c r="G12" s="45"/>
+      <c r="B12" s="49"/>
+      <c r="C12" s="47"/>
+      <c r="D12" s="47"/>
+      <c r="E12" s="47"/>
+      <c r="F12" s="47"/>
+      <c r="G12" s="47"/>
     </row>
     <row r="13" spans="1:26" ht="36" customHeight="1">
-      <c r="A13" s="55"/>
+      <c r="A13" s="50"/>
       <c r="B13" s="39"/>
       <c r="C13" s="39"/>
       <c r="D13" s="39"/>
@@ -2397,39 +2397,39 @@
       <c r="G13" s="39"/>
     </row>
     <row r="14" spans="1:26" ht="37.5" customHeight="1">
-      <c r="A14" s="48" t="s">
+      <c r="A14" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="B14" s="43"/>
-      <c r="C14" s="50" t="s">
+      <c r="B14" s="52"/>
+      <c r="C14" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="D14" s="50" t="s">
+      <c r="D14" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="E14" s="50" t="s">
+      <c r="E14" s="56" t="s">
         <v>63</v>
       </c>
-      <c r="F14" s="50" t="s">
+      <c r="F14" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="G14" s="50" t="s">
+      <c r="G14" s="56" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="15" spans="1:26" ht="85.5" customHeight="1" thickBot="1">
-      <c r="A15" s="52">
+      <c r="A15" s="57">
         <v>11</v>
       </c>
-      <c r="B15" s="51"/>
-      <c r="C15" s="51"/>
-      <c r="D15" s="51"/>
-      <c r="E15" s="51"/>
-      <c r="F15" s="51"/>
-      <c r="G15" s="51"/>
+      <c r="B15" s="55"/>
+      <c r="C15" s="55"/>
+      <c r="D15" s="55"/>
+      <c r="E15" s="55"/>
+      <c r="F15" s="55"/>
+      <c r="G15" s="55"/>
     </row>
     <row r="16" spans="1:26" ht="36" customHeight="1">
-      <c r="A16" s="55"/>
+      <c r="A16" s="50"/>
       <c r="B16" s="39"/>
       <c r="C16" s="39"/>
       <c r="D16" s="39"/>
@@ -2438,39 +2438,39 @@
       <c r="G16" s="39"/>
     </row>
     <row r="17" spans="1:7" ht="37.5" customHeight="1">
-      <c r="A17" s="42" t="s">
+      <c r="A17" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="B17" s="43"/>
-      <c r="C17" s="44" t="s">
+      <c r="B17" s="52"/>
+      <c r="C17" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="D17" s="44" t="s">
+      <c r="D17" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="44" t="s">
+      <c r="E17" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="F17" s="44" t="s">
+      <c r="F17" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="G17" s="44" t="s">
+      <c r="G17" s="46" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:7" ht="85.5" customHeight="1" thickBot="1">
-      <c r="A18" s="54">
+      <c r="A18" s="48">
         <v>15</v>
       </c>
-      <c r="B18" s="47"/>
-      <c r="C18" s="45"/>
-      <c r="D18" s="45"/>
-      <c r="E18" s="45"/>
-      <c r="F18" s="45"/>
-      <c r="G18" s="45"/>
+      <c r="B18" s="49"/>
+      <c r="C18" s="47"/>
+      <c r="D18" s="47"/>
+      <c r="E18" s="47"/>
+      <c r="F18" s="47"/>
+      <c r="G18" s="47"/>
     </row>
     <row r="19" spans="1:7" ht="36" customHeight="1">
-      <c r="A19" s="55"/>
+      <c r="A19" s="50"/>
       <c r="B19" s="39"/>
       <c r="C19" s="39"/>
       <c r="D19" s="39"/>
@@ -2479,39 +2479,39 @@
       <c r="G19" s="39"/>
     </row>
     <row r="20" spans="1:7" ht="37.5" customHeight="1">
-      <c r="A20" s="48" t="s">
+      <c r="A20" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="B20" s="43"/>
-      <c r="C20" s="49" t="s">
+      <c r="B20" s="52"/>
+      <c r="C20" s="53" t="s">
         <v>61</v>
       </c>
-      <c r="D20" s="50" t="s">
+      <c r="D20" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="E20" s="50" t="s">
+      <c r="E20" s="56" t="s">
         <v>60</v>
       </c>
-      <c r="F20" s="50" t="s">
+      <c r="F20" s="56" t="s">
         <v>62</v>
       </c>
-      <c r="G20" s="50" t="s">
+      <c r="G20" s="56" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="21" spans="1:7" ht="85.5" customHeight="1" thickBot="1">
-      <c r="A21" s="52">
+      <c r="A21" s="57">
         <v>18</v>
       </c>
-      <c r="B21" s="47"/>
-      <c r="C21" s="45"/>
-      <c r="D21" s="51"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="51"/>
-      <c r="G21" s="51"/>
+      <c r="B21" s="49"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="55"/>
+      <c r="E21" s="55"/>
+      <c r="F21" s="55"/>
+      <c r="G21" s="55"/>
     </row>
     <row r="22" spans="1:7" ht="36" customHeight="1">
-      <c r="A22" s="55"/>
+      <c r="A22" s="50"/>
       <c r="B22" s="39"/>
       <c r="C22" s="39"/>
       <c r="D22" s="39"/>
@@ -2520,132 +2520,132 @@
       <c r="G22" s="39"/>
     </row>
     <row r="23" spans="1:7" ht="37.5" customHeight="1">
-      <c r="A23" s="42" t="s">
+      <c r="A23" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="B23" s="43"/>
-      <c r="C23" s="44" t="s">
+      <c r="B23" s="52"/>
+      <c r="C23" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="D23" s="44" t="s">
+      <c r="D23" s="46" t="s">
         <v>65</v>
       </c>
-      <c r="E23" s="44" t="s">
+      <c r="E23" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="F23" s="44" t="s">
+      <c r="F23" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="G23" s="44" t="s">
+      <c r="G23" s="46" t="s">
         <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:7" ht="85.5" customHeight="1" thickBot="1">
-      <c r="A24" s="46">
+      <c r="A24" s="60">
         <v>22</v>
       </c>
-      <c r="B24" s="47"/>
-      <c r="C24" s="45"/>
-      <c r="D24" s="45"/>
-      <c r="E24" s="45"/>
-      <c r="F24" s="45"/>
-      <c r="G24" s="45"/>
+      <c r="B24" s="49"/>
+      <c r="C24" s="47"/>
+      <c r="D24" s="47"/>
+      <c r="E24" s="47"/>
+      <c r="F24" s="47"/>
+      <c r="G24" s="47"/>
     </row>
     <row r="25" spans="1:7" ht="23.5">
-      <c r="A25" s="53"/>
-      <c r="B25" s="43"/>
-      <c r="C25" s="44"/>
-      <c r="D25" s="44"/>
-      <c r="E25" s="44"/>
-      <c r="F25" s="44"/>
-      <c r="G25" s="44"/>
+      <c r="A25" s="45"/>
+      <c r="B25" s="52"/>
+      <c r="C25" s="46"/>
+      <c r="D25" s="46"/>
+      <c r="E25" s="46"/>
+      <c r="F25" s="46"/>
+      <c r="G25" s="46"/>
     </row>
     <row r="26" spans="1:7" ht="1.5" customHeight="1" thickBot="1">
-      <c r="A26" s="54">
+      <c r="A26" s="48">
         <v>25</v>
       </c>
-      <c r="B26" s="47"/>
-      <c r="C26" s="45"/>
-      <c r="D26" s="45"/>
-      <c r="E26" s="45"/>
-      <c r="F26" s="45"/>
-      <c r="G26" s="45"/>
+      <c r="B26" s="49"/>
+      <c r="C26" s="47"/>
+      <c r="D26" s="47"/>
+      <c r="E26" s="47"/>
+      <c r="F26" s="47"/>
+      <c r="G26" s="47"/>
     </row>
     <row r="27" spans="1:7" ht="31.5" customHeight="1">
-      <c r="A27" s="48" t="s">
+      <c r="A27" s="51" t="s">
         <v>64</v>
       </c>
-      <c r="B27" s="43"/>
-      <c r="C27" s="49" t="s">
+      <c r="B27" s="52"/>
+      <c r="C27" s="53" t="s">
         <v>62</v>
       </c>
-      <c r="D27" s="50" t="s">
+      <c r="D27" s="56" t="s">
         <v>60</v>
       </c>
-      <c r="E27" s="50" t="s">
+      <c r="E27" s="56" t="s">
         <v>61</v>
       </c>
-      <c r="F27" s="50" t="s">
+      <c r="F27" s="56" t="s">
         <v>65</v>
       </c>
-      <c r="G27" s="50" t="s">
+      <c r="G27" s="56" t="s">
         <v>63</v>
       </c>
     </row>
     <row r="28" spans="1:7" ht="92" customHeight="1" thickBot="1">
-      <c r="A28" s="52">
+      <c r="A28" s="57">
         <v>25</v>
       </c>
-      <c r="B28" s="47"/>
-      <c r="C28" s="45"/>
-      <c r="D28" s="51"/>
-      <c r="E28" s="51"/>
-      <c r="F28" s="51"/>
-      <c r="G28" s="51"/>
+      <c r="B28" s="49"/>
+      <c r="C28" s="47"/>
+      <c r="D28" s="55"/>
+      <c r="E28" s="55"/>
+      <c r="F28" s="55"/>
+      <c r="G28" s="55"/>
     </row>
     <row r="29" spans="1:7" ht="17" customHeight="1">
-      <c r="A29" s="40"/>
-      <c r="B29" s="41"/>
-      <c r="C29" s="41"/>
-      <c r="D29" s="41"/>
-      <c r="E29" s="41"/>
-      <c r="F29" s="41"/>
-      <c r="G29" s="41"/>
+      <c r="A29" s="62"/>
+      <c r="B29" s="63"/>
+      <c r="C29" s="63"/>
+      <c r="D29" s="63"/>
+      <c r="E29" s="63"/>
+      <c r="F29" s="63"/>
+      <c r="G29" s="63"/>
     </row>
     <row r="30" spans="1:7" ht="37.5" customHeight="1">
-      <c r="A30" s="42" t="s">
+      <c r="A30" s="58" t="s">
         <v>59</v>
       </c>
-      <c r="B30" s="43"/>
-      <c r="C30" s="44" t="s">
+      <c r="B30" s="52"/>
+      <c r="C30" s="46" t="s">
         <v>61</v>
       </c>
-      <c r="D30" s="44" t="s">
+      <c r="D30" s="46" t="s">
         <v>66</v>
       </c>
-      <c r="E30" s="44" t="s">
+      <c r="E30" s="46" t="s">
         <v>60</v>
       </c>
-      <c r="F30" s="44" t="s">
+      <c r="F30" s="46" t="s">
         <v>62</v>
       </c>
-      <c r="G30" s="44" t="s">
+      <c r="G30" s="46" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="31" spans="1:7" ht="85.5" customHeight="1" thickBot="1">
-      <c r="A31" s="46">
+      <c r="A31" s="60">
         <v>29</v>
       </c>
-      <c r="B31" s="47"/>
-      <c r="C31" s="45"/>
-      <c r="D31" s="45"/>
-      <c r="E31" s="45"/>
-      <c r="F31" s="45"/>
-      <c r="G31" s="45"/>
+      <c r="B31" s="49"/>
+      <c r="C31" s="47"/>
+      <c r="D31" s="47"/>
+      <c r="E31" s="47"/>
+      <c r="F31" s="47"/>
+      <c r="G31" s="47"/>
     </row>
     <row r="32" spans="1:7" ht="30.5" customHeight="1">
-      <c r="B32" s="38" t="s">
+      <c r="B32" s="61" t="s">
         <v>4</v>
       </c>
       <c r="C32" s="39"/>
@@ -3620,11 +3620,69 @@
     <row r="997" customFormat="1" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="83">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="F1:G1"/>
-    <mergeCell ref="A2:G2"/>
-    <mergeCell ref="A3:B3"/>
-    <mergeCell ref="A4:G4"/>
+    <mergeCell ref="B32:F32"/>
+    <mergeCell ref="A29:G29"/>
+    <mergeCell ref="A30:B30"/>
+    <mergeCell ref="C30:C31"/>
+    <mergeCell ref="D30:D31"/>
+    <mergeCell ref="E30:E31"/>
+    <mergeCell ref="F30:F31"/>
+    <mergeCell ref="G30:G31"/>
+    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="G27:G28"/>
+    <mergeCell ref="A28:B28"/>
+    <mergeCell ref="A25:B25"/>
+    <mergeCell ref="C25:C26"/>
+    <mergeCell ref="D25:D26"/>
+    <mergeCell ref="E25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="A26:B26"/>
+    <mergeCell ref="A27:B27"/>
+    <mergeCell ref="C27:C28"/>
+    <mergeCell ref="D27:D28"/>
+    <mergeCell ref="E27:E28"/>
+    <mergeCell ref="F27:F28"/>
+    <mergeCell ref="A22:G22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="C23:C24"/>
+    <mergeCell ref="D23:D24"/>
+    <mergeCell ref="E23:E24"/>
+    <mergeCell ref="F23:F24"/>
+    <mergeCell ref="G23:G24"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="C20:C21"/>
+    <mergeCell ref="D20:D21"/>
+    <mergeCell ref="E20:E21"/>
+    <mergeCell ref="F20:F21"/>
+    <mergeCell ref="G20:G21"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A17:B17"/>
+    <mergeCell ref="C17:C18"/>
+    <mergeCell ref="D17:D18"/>
+    <mergeCell ref="E17:E18"/>
+    <mergeCell ref="F17:F18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="A18:B18"/>
+    <mergeCell ref="A13:G13"/>
+    <mergeCell ref="A14:B14"/>
+    <mergeCell ref="C14:C15"/>
+    <mergeCell ref="D14:D15"/>
+    <mergeCell ref="E14:E15"/>
+    <mergeCell ref="F14:F15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="A15:B15"/>
+    <mergeCell ref="A10:G10"/>
+    <mergeCell ref="A11:B11"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="F11:F12"/>
+    <mergeCell ref="G11:G12"/>
+    <mergeCell ref="A12:B12"/>
     <mergeCell ref="G5:G6"/>
     <mergeCell ref="A6:B6"/>
     <mergeCell ref="A7:G7"/>
@@ -3640,69 +3698,11 @@
     <mergeCell ref="D5:D6"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="F5:F6"/>
-    <mergeCell ref="A10:G10"/>
-    <mergeCell ref="A11:B11"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="F11:F12"/>
-    <mergeCell ref="G11:G12"/>
-    <mergeCell ref="A12:B12"/>
-    <mergeCell ref="A13:G13"/>
-    <mergeCell ref="A14:B14"/>
-    <mergeCell ref="C14:C15"/>
-    <mergeCell ref="D14:D15"/>
-    <mergeCell ref="E14:E15"/>
-    <mergeCell ref="F14:F15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="A15:B15"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A17:B17"/>
-    <mergeCell ref="C17:C18"/>
-    <mergeCell ref="D17:D18"/>
-    <mergeCell ref="E17:E18"/>
-    <mergeCell ref="F17:F18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="A18:B18"/>
-    <mergeCell ref="A19:G19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="C20:C21"/>
-    <mergeCell ref="D20:D21"/>
-    <mergeCell ref="E20:E21"/>
-    <mergeCell ref="F20:F21"/>
-    <mergeCell ref="G20:G21"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:G22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="C23:C24"/>
-    <mergeCell ref="D23:D24"/>
-    <mergeCell ref="E23:E24"/>
-    <mergeCell ref="F23:F24"/>
-    <mergeCell ref="G23:G24"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="G27:G28"/>
-    <mergeCell ref="A28:B28"/>
-    <mergeCell ref="A25:B25"/>
-    <mergeCell ref="C25:C26"/>
-    <mergeCell ref="D25:D26"/>
-    <mergeCell ref="E25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="A26:B26"/>
-    <mergeCell ref="A27:B27"/>
-    <mergeCell ref="C27:C28"/>
-    <mergeCell ref="D27:D28"/>
-    <mergeCell ref="E27:E28"/>
-    <mergeCell ref="F27:F28"/>
-    <mergeCell ref="B32:F32"/>
-    <mergeCell ref="A29:G29"/>
-    <mergeCell ref="A30:B30"/>
-    <mergeCell ref="C30:C31"/>
-    <mergeCell ref="D30:D31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="F30:F31"/>
-    <mergeCell ref="G30:G31"/>
-    <mergeCell ref="A31:B31"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="F1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A3:B3"/>
+    <mergeCell ref="A4:G4"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <drawing r:id="rId1"/>

</xml_diff>